<commit_message>
feat: nine site x tier growth factors and optional site location
- Growth factors are now 3 site categories x growth tiers 1-3 (9 values)
  instead of 3 x tree/shrub (6). Each species has a tier per category
  (SPECIES_GROWTH_TIERS, default 1); the tier factor scales stored annual
  increments and, for records without increments, the assumed 2% rate.
  Legacy six-factor files map to tiers 1 and 2.
- Library manager: tier 1/2/3 factor inputs per category tab and an
  editable "growth tier" column (1/2/3 dropdown) with validation.
- Sites take an optional latitude/longitude: add-site dialog, banner with
  map link and edit, data workbook columns, comparison sheet columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/presets/ForeCarb_데이터_예시.xlsx
+++ b/presets/ForeCarb_데이터_예시.xlsx
@@ -19,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -66,11 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -438,13 +441,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +473,16 @@
           <t>대상지 유형</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>위도</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>경도</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -486,6 +501,12 @@
           <t>산불피해지 자연복원</t>
         </is>
       </c>
+      <c r="E2" s="2" t="n">
+        <v>36.4986</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>127.2896</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -539,6 +560,12 @@
         <is>
           <t>산불피해지 자연복원</t>
         </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>36.4986</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>127.2896</v>
       </c>
     </row>
   </sheetData>
@@ -560,7 +587,7 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -2886,92 +2913,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ForeCarb 입력 데이터 양식</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr"/>
+      <c r="A2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>1. [지역] 시트: 지역명, 가로·세로(m), 대상지 유형을 적습니다. 지역마다 탭이 하나씩 만들어집니다.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   위도·경도는 선택 입력입니다 (십진수 도, 예: 36.4986 / 127.2896). 둘 다 적으면 지역 위치로 표시됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>2. [수종] 시트: 한 줄에 한 수종(같은 직경·생존율 묶음)을 적습니다. 지역명은 [지역] 시트와 같아야 합니다.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>3. 구분은 교목 또는 관목, 수종은 [수종목록] 시트의 이름(국명 또는 학명)을 그대로 씁니다.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>4. 직경은 cm 단위입니다 (교목 DBH, 관목 RCD). 적합 직경범위 밖의 행은 계산에서 제외됩니다.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>5. 현재 생존율(%)은 0년차 수량에, 연간 생존율(%)은 해마다 누적 적용됩니다: N(t) = N × 현재 생존율 × 연간 생존율^t</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   비워 두면 100 %(전량 생존)이며, 기존 결과(전량 생존)와 생존률 반영 결과가 함께 표시됩니다.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>6. 두 번째 변수는 수고·임분밀도 등 보조변수가 필요한 식에만 적습니다 (비우면 기본값).</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>7. ForeCarb 메뉴 [파일] → [데이터 불러오기] 로 불러오면 지역 탭이 만들어지고 바로 계산됩니다.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>8. [파일] → [데이터 저장] 은 지금 열린 지역들의 입력을 이 양식으로 저장합니다.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>예시 데이터는 최종보고서 표3의 Profile 1~3 (400 m²) 입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Profile 1 의 위도·경도는 입력 방법을 보여 주기 위한 예시 좌표(국립세종수목원 부근)입니다.</t>
         </is>
       </c>
     </row>

</xml_diff>